<commit_message>
20260511 : 현재 local과 repository 일치화 하기 위한 작업
</commit_message>
<xml_diff>
--- a/Python_2026/JRCM_KPI_2026.xlsx
+++ b/Python_2026/JRCM_KPI_2026.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Development_2026\Python_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{92C751C3-7D43-4ADA-BCF4-65ECA43441B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5209EA93-B9D3-4E79-A65D-B414D61DCBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{11C83BD3-EFE0-40C3-BAD3-524289020AF7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{11C83BD3-EFE0-40C3-BAD3-524289020AF7}"/>
   </bookViews>
   <sheets>
     <sheet name="export" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentManualCount="12"/>
+  <calcPr calcId="191029" concurrentManualCount="12"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
   <si>
     <t>Item</t>
   </si>
@@ -41,14 +54,6 @@
   </si>
   <si>
     <t>Very High</t>
-  </si>
-  <si>
-    <t>0 cases(100%): 2.5
-1-2 cases : -0.5
-3-5 cases: Story point -1
-6-9 cases: Story point -1.5
-10-12 cases: Story point -2
-&lt;13 cases: Story point -2.5</t>
   </si>
   <si>
     <t>Job Status update
@@ -56,13 +61,6 @@
   </si>
   <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>0 cases(100%): 2
-1-2 cases : -0.5
-3-5 cases: Story point -1
-6-9 cases: Story point -1.5
-&lt;10 cases: Story point -2</t>
   </si>
   <si>
     <t>Resource issue for tasks mentioned in RFQ</t>
@@ -77,12 +75,6 @@
   </si>
   <si>
     <t>Mid</t>
-  </si>
-  <si>
-    <t>All achieved (100%): 1.5
-1-2 cases : -0.5
-3-5 cases: Story point -1
-&lt;6 cases: Story point -1.5</t>
   </si>
   <si>
     <t>KPM Ticket rules
@@ -97,15 +89,6 @@
     <t>Free testing</t>
   </si>
   <si>
-    <t>0 cases(100%): 2.5
-No Free test: 0
-1-2 cases : -0.5
-3-5 cases: Story point -1
-6-9 cases: Story point -1.5
-10-12 cases: Story point -2
-&lt;13 cases: Story point -2.5</t>
-  </si>
-  <si>
     <t>May (Count)</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -207,6 +190,43 @@
   <si>
     <t>Value (Max 16.5 point) - Target 100%</t>
     <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>All achieved (100%): 0
+1-2 cases : 0.5
+3-5 cases: Story point : 1
+6-9 cases: Story point : 1.5
+10-12 cases: Story point : 2
+&lt;13 cases: Story point : 2.5</t>
+  </si>
+  <si>
+    <t>All achieved (100%): 0
+1-2 cases : 0.5
+3-5 cases: Story point :1
+6-9 cases: Story point : 1.5
+&lt;10 cases: Story point : 2</t>
+  </si>
+  <si>
+    <t>All achieved (100%): 0
+1-2 cases : 0.5
+3-5 cases: Story point 1
+&lt;6 cases: Story point 1.5</t>
+  </si>
+  <si>
+    <t>All achieved (100%): 0
+1-2 cases : 0.5
+3-5 cases: Story point : 1
+6-9 cases: Story point : 1.5
+&lt;10 cases: Story point : 2</t>
+  </si>
+  <si>
+    <t>All achieved (100%): 0
+1-2 cases : 0.5
+3-5 cases: Story point : 1
+6-9 cases: Story point : 1.5
+10-12 cases: Story point : 2
+&lt;13 cases: Story point : 2.5
+or 0 cases: 2.5</t>
   </si>
 </sst>
 </file>
@@ -826,7 +846,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -857,14 +877,17 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -940,6 +963,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR"/>
+              <a:t>KPI Measurement - JRCM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1114,7 +1162,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7058823529411764E-2</c:v>
+                  <c:v>7.0588235294117646E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1260,16 +1308,16 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="1">
-                  <c:v>0.51515151515151514</c:v>
+                  <c:v>0.93939393939393945</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.84848484848484851</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>0.87878787878787878</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.84848484848484851</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1476,7 +1524,930 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR"/>
+              <a:t>KPI Count monthly</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ko-KR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="15"/>
+      <c:rotY val="20"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="1"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:bar3DChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>export!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Jan (Count)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="ko-KR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>export!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Job Status update
+repoting of general blockers/ job stoppers</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Resource issue for tasks mentioned in RFQ</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Follow up guidelines for tasks &amp; release note for testing
+- Maintenance activity not following general process
+ - Following test car usage PI</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>All the information and knowledge what we provided and working log, specification should be kept and trained internally</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>KPM Ticket rules
+ - KPM Ticket creation
+ - KPM Check-back
+ - KPM Verification</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>KPM ticket quality</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Free testing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>export!$F$2:$F$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5D46-4927-BEE1-D72297392324}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>export!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Feb (Count)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>export!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Job Status update
+repoting of general blockers/ job stoppers</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Resource issue for tasks mentioned in RFQ</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Follow up guidelines for tasks &amp; release note for testing
+- Maintenance activity not following general process
+ - Following test car usage PI</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>All the information and knowledge what we provided and working log, specification should be kept and trained internally</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>KPM Ticket rules
+ - KPM Ticket creation
+ - KPM Check-back
+ - KPM Verification</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>KPM ticket quality</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Free testing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>export!$H$2:$H$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5D46-4927-BEE1-D72297392324}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>export!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mar(Count)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="ko-KR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>export!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Job Status update
+repoting of general blockers/ job stoppers</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Resource issue for tasks mentioned in RFQ</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Follow up guidelines for tasks &amp; release note for testing
+- Maintenance activity not following general process
+ - Following test car usage PI</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>All the information and knowledge what we provided and working log, specification should be kept and trained internally</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>KPM Ticket rules
+ - KPM Ticket creation
+ - KPM Check-back
+ - KPM Verification</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>KPM ticket quality</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Free testing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>export!$J$2:$J$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-5D46-4927-BEE1-D72297392324}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>export!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Apr(Count)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="ko-KR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>export!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Job Status update
+repoting of general blockers/ job stoppers</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Resource issue for tasks mentioned in RFQ</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Follow up guidelines for tasks &amp; release note for testing
+- Maintenance activity not following general process
+ - Following test car usage PI</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>All the information and knowledge what we provided and working log, specification should be kept and trained internally</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>KPM Ticket rules
+ - KPM Ticket creation
+ - KPM Check-back
+ - KPM Verification</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>KPM ticket quality</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Free testing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>export!$L$2:$L$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-5D46-4927-BEE1-D72297392324}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:shape val="box"/>
+        <c:axId val="105181056"/>
+        <c:axId val="105177696"/>
+        <c:axId val="0"/>
+      </c:bar3DChart>
+      <c:catAx>
+        <c:axId val="105181056"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ko-KR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="105177696"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="105177696"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ko-KR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="105181056"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ko-KR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="ko-KR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1987,6 +2958,500 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="286">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -2052,6 +3517,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>136071</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>326571</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>54429</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>68036</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD914C14-77B3-C607-3346-3DDE91E40664}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2403,76 +3904,76 @@
         <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="P1" s="4" t="s">
+      <c r="U1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="W1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="X1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="T1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>29</v>
-      </c>
       <c r="AC1" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="99" x14ac:dyDescent="0.3">
@@ -2482,8 +3983,8 @@
       <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>7</v>
+      <c r="C2" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="D2" s="3">
         <v>2.5</v>
@@ -2495,36 +3996,36 @@
         <v>2</v>
       </c>
       <c r="G2" s="3">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="H2" s="3">
         <v>0</v>
       </c>
       <c r="I2" s="3">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
         <v>1</v>
       </c>
       <c r="K2" s="3">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="L2" s="3">
         <v>0</v>
       </c>
       <c r="M2" s="3">
-        <v>2.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>10</v>
+      <c r="C3" s="13" t="s">
+        <v>47</v>
       </c>
       <c r="D3" s="3">
         <v>2</v>
@@ -2536,36 +4037,36 @@
         <v>0</v>
       </c>
       <c r="G3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H3" s="3">
         <v>0</v>
       </c>
       <c r="I3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3">
         <v>0</v>
       </c>
       <c r="K3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <v>0</v>
       </c>
       <c r="M3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>47</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
@@ -2577,36 +4078,36 @@
         <v>0</v>
       </c>
       <c r="G4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
       </c>
       <c r="I4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3">
         <v>0</v>
       </c>
       <c r="K4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L4" s="3">
         <v>0</v>
       </c>
       <c r="M4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>47</v>
       </c>
       <c r="D5" s="3">
         <v>2</v>
@@ -2618,36 +4119,36 @@
         <v>1</v>
       </c>
       <c r="G5" s="3">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3">
         <v>4</v>
       </c>
       <c r="K5" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L5" s="3">
         <v>0</v>
       </c>
       <c r="M5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="66" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>48</v>
       </c>
       <c r="D6" s="3">
         <v>1.5</v>
@@ -2659,36 +4160,36 @@
         <v>0</v>
       </c>
       <c r="G6" s="3">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
       </c>
       <c r="K6" s="3">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3">
         <v>0</v>
       </c>
       <c r="M6" s="3">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="D7" s="3">
         <v>2</v>
@@ -2700,36 +4201,36 @@
         <v>0</v>
       </c>
       <c r="G7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3">
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
       </c>
       <c r="K7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3">
         <v>0</v>
       </c>
       <c r="M7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="D8" s="3">
         <v>2</v>
@@ -2741,36 +4242,36 @@
         <v>1</v>
       </c>
       <c r="G8" s="3">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3">
         <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3">
         <v>1</v>
       </c>
       <c r="K8" s="3">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="L8" s="3">
         <v>0</v>
       </c>
       <c r="M8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>19</v>
+      <c r="C9" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="D9" s="3">
         <v>2.5</v>
@@ -2782,13 +4283,13 @@
         <v>0</v>
       </c>
       <c r="G9" s="3">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3">
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -2806,7 +4307,7 @@
     <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3">
         <v>85</v>
@@ -2818,28 +4319,36 @@
         <v>16.5</v>
       </c>
       <c r="F10" s="3">
+        <f>SUM(F2:F9)</f>
         <v>4</v>
       </c>
       <c r="G10" s="3">
-        <v>8.5</v>
+        <f>SUM(G2:G9)</f>
+        <v>1</v>
       </c>
       <c r="H10" s="3">
+        <f>SUM(H2:H9)</f>
         <v>0</v>
       </c>
       <c r="I10" s="3">
-        <v>14</v>
+        <f>SUM(I2:I9)</f>
+        <v>0</v>
       </c>
       <c r="J10" s="3">
-        <v>4</v>
+        <f>SUM(J2:J9)</f>
+        <v>6</v>
       </c>
       <c r="K10" s="3">
-        <v>5.5</v>
+        <f>SUM(K2:K9)</f>
+        <v>2</v>
       </c>
       <c r="L10" s="3">
+        <f>SUM(L2:L9)</f>
         <v>0</v>
       </c>
       <c r="M10" s="3">
-        <v>14</v>
+        <f>SUM(M2:M9)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.3">
@@ -2848,84 +4357,84 @@
         <v>4.7058823529411764E-2</v>
       </c>
       <c r="G11" s="8">
-        <f>(G10/$D$10)</f>
-        <v>0.51515151515151514</v>
+        <f>1-(G10/$D$10)</f>
+        <v>0.93939393939393945</v>
       </c>
       <c r="H11" s="8">
         <f>(H10/$C$10)</f>
         <v>0</v>
       </c>
       <c r="I11" s="8">
-        <f>(I10/$D$10)</f>
-        <v>0.84848484848484851</v>
+        <f>1-(I10/$D$10)</f>
+        <v>1</v>
       </c>
       <c r="J11" s="8">
         <f>(J10/$C$10)</f>
-        <v>4.7058823529411764E-2</v>
+        <v>7.0588235294117646E-2</v>
       </c>
       <c r="K11" s="8">
-        <f>(K10/$D$10)</f>
-        <v>0.33333333333333331</v>
+        <f>1-(K10/$D$10)</f>
+        <v>0.87878787878787878</v>
       </c>
       <c r="L11" s="8">
         <f>(L10/$C$10)</f>
         <v>0</v>
       </c>
       <c r="M11" s="8">
-        <f>(M10/$D$10)</f>
-        <v>0.84848484848484851</v>
+        <f>1-(M10/$D$10)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="C13" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10" t="s">
+      <c r="C13" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="J13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="K13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="L13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="M13" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="N13" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="O13" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="P13" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="Q13" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="C14" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="11"/>
+      <c r="C14" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="12"/>
       <c r="E14" s="8">
         <f>(F10/$C$10)</f>
         <v>4.7058823529411764E-2</v>
@@ -2936,7 +4445,7 @@
       </c>
       <c r="G14" s="8">
         <f>(J10/$C$10)</f>
-        <v>4.7058823529411764E-2</v>
+        <v>7.0588235294117646E-2</v>
       </c>
       <c r="H14" s="8">
         <f>(L10/$C$10)</f>
@@ -2950,31 +4459,31 @@
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="5"/>
-      <c r="Q14" s="12">
+      <c r="Q14" s="10">
         <f>AVERAGE(E14:P14)</f>
-        <v>2.3529411764705882E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="C15" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="11"/>
+      <c r="C15" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="12"/>
       <c r="E15" s="8">
-        <f>(G10/$D$10)</f>
-        <v>0.51515151515151514</v>
+        <f>G11</f>
+        <v>0.93939393939393945</v>
       </c>
       <c r="F15" s="8">
-        <f>(I10/$D$10)</f>
-        <v>0.84848484848484851</v>
+        <f>I11</f>
+        <v>1</v>
       </c>
       <c r="G15" s="8">
-        <f>(K10/$D$10)</f>
-        <v>0.33333333333333331</v>
+        <f>K11</f>
+        <v>0.87878787878787878</v>
       </c>
       <c r="H15" s="8">
-        <f>(M10/$D$10)</f>
-        <v>0.84848484848484851</v>
+        <f>M11</f>
+        <v>1</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
@@ -2984,9 +4493,9 @@
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="5"/>
-      <c r="Q15" s="12">
+      <c r="Q15" s="10">
         <f>AVERAGE(E15:P15)</f>
-        <v>0.63636363636363635</v>
+        <v>0.95454545454545459</v>
       </c>
     </row>
   </sheetData>
@@ -2997,10 +4506,11 @@
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_</oddHeader>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>